<commit_message>
Update Material Master (06.10.2026)
</commit_message>
<xml_diff>
--- a/Excel/main template/ERSA.xlsx
+++ b/Excel/main template/ERSA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DANIEL\ANTIGRAVITY\MASTER DATA GOVERNANCE\MATERIAL MASTER\Excel\main template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32755071-C3A1-49B7-8533-ECD1B5CE9597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7721C5C8-5AFD-49AD-89FD-9EDD1A156C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E3D08ABF-0C41-493A-BD8B-FB6623B75271}"/>
   </bookViews>
@@ -39,12 +39,6 @@
     <t>F</t>
   </si>
   <si>
-    <t>ERSA</t>
-  </si>
-  <si>
-    <t>ESP027</t>
-  </si>
-  <si>
     <t>PAC</t>
   </si>
   <si>
@@ -508,13 +502,19 @@
   </si>
   <si>
     <t>04</t>
+  </si>
+  <si>
+    <t>OSS008</t>
+  </si>
+  <si>
+    <t>ZOS3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,6 +538,19 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -575,12 +588,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -590,6 +603,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -909,6 +926,7 @@
   <dimension ref="A1:ED2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
+    <col min="1" max="1" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="34.6328125" bestFit="1" customWidth="1"/>
@@ -917,428 +935,428 @@
   <sheetData>
     <row r="1" spans="1:134" s="4" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="W1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="Y1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="Z1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="Y1" s="3" t="s">
+      <c r="AA1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="Z1" s="3" t="s">
+      <c r="AB1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="AA1" s="3" t="s">
+      <c r="AC1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="AB1" s="3" t="s">
+      <c r="AD1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="AC1" s="3" t="s">
+      <c r="AE1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="AD1" s="3" t="s">
+      <c r="AF1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="AE1" s="3" t="s">
+      <c r="AG1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="AH1" s="3" t="s">
+      <c r="AJ1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="AI1" s="3" t="s">
+      <c r="AK1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="AJ1" s="3" t="s">
+      <c r="AL1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="AK1" s="3" t="s">
+      <c r="AM1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="AL1" s="3" t="s">
+      <c r="AN1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="AM1" s="3" t="s">
+      <c r="AO1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="AN1" s="3" t="s">
+      <c r="AP1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="AO1" s="3" t="s">
+      <c r="AQ1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="AP1" s="3" t="s">
+      <c r="AR1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="AQ1" s="3" t="s">
+      <c r="AS1" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="AR1" s="3" t="s">
+      <c r="AT1" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="AS1" s="3" t="s">
+      <c r="AU1" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="AT1" s="3" t="s">
+      <c r="AV1" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="AU1" s="3" t="s">
+      <c r="AW1" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="AV1" s="3" t="s">
+      <c r="AX1" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="AW1" s="3" t="s">
+      <c r="AY1" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AZ1" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="AY1" s="3" t="s">
+      <c r="BA1" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="AZ1" s="3" t="s">
+      <c r="BB1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="BA1" s="3" t="s">
+      <c r="BC1" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="BB1" s="3" t="s">
+      <c r="BD1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="BC1" s="3" t="s">
+      <c r="BE1" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="BD1" s="3" t="s">
+      <c r="BF1" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="BE1" s="3" t="s">
+      <c r="BG1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="BF1" s="3" t="s">
+      <c r="BH1" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="BG1" s="3" t="s">
+      <c r="BI1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="BH1" s="3" t="s">
+      <c r="BJ1" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="BI1" s="3" t="s">
+      <c r="BK1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="BJ1" s="3" t="s">
+      <c r="BL1" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="BK1" s="3" t="s">
+      <c r="BM1" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="BL1" s="3" t="s">
+      <c r="BN1" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="BM1" s="3" t="s">
+      <c r="BO1" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="BN1" s="3" t="s">
+      <c r="BP1" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="BO1" s="3" t="s">
+      <c r="BQ1" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="BP1" s="3" t="s">
+      <c r="BR1" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="BQ1" s="3" t="s">
+      <c r="BS1" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="BR1" s="3" t="s">
+      <c r="BT1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="BS1" s="3" t="s">
+      <c r="BU1" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="BT1" s="3" t="s">
+      <c r="BV1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="BU1" s="3" t="s">
+      <c r="BW1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="BV1" s="3" t="s">
+      <c r="BX1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="BW1" s="3" t="s">
+      <c r="BY1" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="BX1" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="BY1" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="BZ1" s="3"/>
       <c r="CA1" s="3"/>
       <c r="CB1" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="CC1" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="CD1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="CC1" s="3" t="s">
+      <c r="CE1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="CD1" s="3" t="s">
+      <c r="CF1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="CE1" s="3" t="s">
+      <c r="CG1" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="CF1" s="3" t="s">
+      <c r="CH1" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="CG1" s="3" t="s">
+      <c r="CI1" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="CH1" s="3" t="s">
+      <c r="CJ1" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="CI1" s="3" t="s">
+      <c r="CK1" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="CJ1" s="3" t="s">
+      <c r="CL1" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="CK1" s="3" t="s">
+      <c r="CM1" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="CL1" s="3" t="s">
+      <c r="CN1" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="CM1" s="3" t="s">
+      <c r="CO1" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="CN1" s="3" t="s">
+      <c r="CP1" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="CO1" s="3" t="s">
+      <c r="CQ1" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="CP1" s="3" t="s">
+      <c r="CR1" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="CQ1" s="3" t="s">
+      <c r="CS1" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="CR1" s="3" t="s">
+      <c r="CT1" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="CS1" s="3" t="s">
+      <c r="CU1" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="CT1" s="3" t="s">
+      <c r="CV1" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="CU1" s="3" t="s">
+      <c r="CW1" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="CV1" s="3" t="s">
+      <c r="CX1" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="CW1" s="3" t="s">
+      <c r="CY1" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="CX1" s="3" t="s">
+      <c r="CZ1" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="CY1" s="3" t="s">
+      <c r="DA1" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="CZ1" s="3" t="s">
+      <c r="DB1" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="DA1" s="3" t="s">
+      <c r="DC1" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="DB1" s="3" t="s">
+      <c r="DD1" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="DC1" s="3" t="s">
+      <c r="DE1" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="DD1" s="3" t="s">
+      <c r="DF1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="DE1" s="3" t="s">
+      <c r="DG1" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="DF1" s="3" t="s">
+      <c r="DH1" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="DG1" s="3" t="s">
+      <c r="DI1" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="DH1" s="3" t="s">
+      <c r="DJ1" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="DI1" s="3" t="s">
+      <c r="DK1" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="DJ1" s="3" t="s">
+      <c r="DL1" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="DK1" s="3" t="s">
+      <c r="DM1" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="DL1" s="3" t="s">
+      <c r="DN1" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="DM1" s="3" t="s">
+      <c r="DO1" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="DN1" s="3" t="s">
+      <c r="DP1" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="DO1" s="3" t="s">
+      <c r="DQ1" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="DP1" s="3" t="s">
+      <c r="DR1" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="DQ1" s="3" t="s">
+      <c r="DS1" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="DR1" s="3" t="s">
+      <c r="DT1" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="DS1" s="3" t="s">
+      <c r="DU1" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="DT1" s="3" t="s">
+      <c r="DV1" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="DU1" s="3" t="s">
+      <c r="DW1" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="DV1" s="3" t="s">
+      <c r="DX1" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="DW1" s="3" t="s">
+      <c r="DY1" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="DX1" s="3" t="s">
+      <c r="DZ1" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="DY1" s="3" t="s">
+      <c r="EA1" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="DZ1" s="3" t="s">
+      <c r="EB1" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="EA1" s="3" t="s">
+      <c r="EC1" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="EB1" s="3" t="s">
+      <c r="ED1" s="3" t="s">
         <v>154</v>
-      </c>
-      <c r="EC1" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="ED1" s="3" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:134" s="2" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
-        <v>60009458</v>
+      <c r="A2" s="7">
+        <v>50001540</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>4</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="N2" s="5">
         <v>1200</v>
@@ -1350,58 +1368,58 @@
         <v>1</v>
       </c>
       <c r="T2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="V2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="U2" s="2" t="s">
+      <c r="W2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="AD2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="V2" s="2" t="s">
+      <c r="AE2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="AF2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="W2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="X2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="AD2" s="1" t="s">
+      <c r="AH2" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="AE2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="AF2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="AH2" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="AI2" s="2">
         <v>200201</v>
       </c>
       <c r="AJ2" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="AM2" s="2">
         <v>1</v>
       </c>
       <c r="AN2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="BA2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="BG2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="BA2" s="2" t="s">
+      <c r="BH2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="BG2" s="2" t="s">
+      <c r="BI2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="BH2" s="2" t="s">
+      <c r="BJ2" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="BI2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="BJ2" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="BN2" s="2" t="s">
         <v>0</v>
@@ -1410,16 +1428,16 @@
         <v>1</v>
       </c>
       <c r="BT2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="BZ2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="CA2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="BZ2" s="2" t="s">
+      <c r="CB2" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="CA2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="CB2" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="CD2" s="2">
         <v>2</v>
@@ -1428,32 +1446,32 @@
         <v>1207</v>
       </c>
       <c r="CJ2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="CK2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="CL2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="CM2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="CN2" s="2">
         <v>100</v>
       </c>
       <c r="CP2" s="1"/>
       <c r="CQ2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="CS2" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="CS2" s="2" t="s">
-        <v>12</v>
       </c>
       <c r="CV2" s="2">
         <v>1000</v>
       </c>
       <c r="CY2" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>